<commit_message>
Build core CRDQE engine with validation pipeline and Excel reporting
</commit_message>
<xml_diff>
--- a/data/output/cleaned/cleaned_data.xlsx
+++ b/data/output/cleaned/cleaned_data.xlsx
@@ -28886,8 +28886,10 @@
     <row r="413"/>
     <row r="414"/>
     <row r="415">
-      <c r="I415" t="n">
-        <v>574</v>
+      <c r="I415" t="inlineStr">
+        <is>
+          <t>574</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>